<commit_message>
CPM download model fix.
</commit_message>
<xml_diff>
--- a/api/static/cpm.xlsx
+++ b/api/static/cpm.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anama\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b808ff425a94bbdc/Documents/Faculdade/Iniciação Científica/ARNA_UFPE/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27ADA2EC-15F6-4E20-8CEE-C19BC5F93D3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{27ADA2EC-15F6-4E20-8CEE-C19BC5F93D3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{133F4A08-ECB9-4EC8-8AD5-CACDE2D662D6}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7EB555F7-2C2B-4388-8B33-737FD34076B1}"/>
   </bookViews>
@@ -71,10 +71,10 @@
     <t>G</t>
   </si>
   <si>
-    <t>D, E</t>
-  </si>
-  <si>
-    <t>G, H</t>
+    <t>G,H</t>
+  </si>
+  <si>
+    <t>D,E</t>
   </si>
 </sst>
 </file>
@@ -619,7 +619,7 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C8">
         <v>8</v>
@@ -657,7 +657,7 @@
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10">
         <v>0</v>

</xml_diff>

<commit_message>
Standardize xlsx input (MC).
</commit_message>
<xml_diff>
--- a/api/static/cpm.xlsx
+++ b/api/static/cpm.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b808ff425a94bbdc/Documents/Faculdade/Iniciação Científica/ARNA_UFPE/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anama\OneDrive\Documents\Faculdade\Iniciação Científica\ARNA_UFPE\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{27ADA2EC-15F6-4E20-8CEE-C19BC5F93D3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{133F4A08-ECB9-4EC8-8AD5-CACDE2D662D6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC46E3F5-F664-4DB2-9938-BBB7F5817892}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7EB555F7-2C2B-4388-8B33-737FD34076B1}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="15">
   <si>
     <t>Precedentes</t>
   </si>
@@ -71,10 +71,13 @@
     <t>G</t>
   </si>
   <si>
-    <t>G,H</t>
-  </si>
-  <si>
-    <t>D,E</t>
+    <t>inicio</t>
+  </si>
+  <si>
+    <t>D, E</t>
+  </si>
+  <si>
+    <t>G, H</t>
   </si>
 </sst>
 </file>
@@ -505,10 +508,10 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
@@ -521,13 +524,13 @@
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
@@ -540,13 +543,13 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
       </c>
       <c r="C4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
@@ -559,13 +562,13 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5">
         <v>4</v>
-      </c>
-      <c r="C5">
-        <v>5</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -578,13 +581,13 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
       </c>
       <c r="C6">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
@@ -597,13 +600,13 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
@@ -616,13 +619,13 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C8">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
@@ -635,13 +638,13 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C9">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
@@ -654,13 +657,13 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
@@ -672,9 +675,15 @@
       <c r="U10" s="3"/>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
+      <c r="A11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>

</xml_diff>

<commit_message>
Update model .xlsx folder, standardize activity name input.
</commit_message>
<xml_diff>
--- a/api/static/cpm.xlsx
+++ b/api/static/cpm.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anama\OneDrive\Documents\Faculdade\Iniciação Científica\ARNA_UFPE\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC46E3F5-F664-4DB2-9938-BBB7F5817892}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D29A10A-EE16-4A9E-83F3-8888B43A69E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7EB555F7-2C2B-4388-8B33-737FD34076B1}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
   <si>
     <t>Precedentes</t>
   </si>
@@ -44,40 +44,16 @@
     <t>fim</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
     <t>Duracao</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>E</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>H</t>
-  </si>
-  <si>
-    <t>G</t>
   </si>
   <si>
     <t>inicio</t>
   </si>
   <si>
-    <t>D, E</t>
+    <t>4, 5</t>
   </si>
   <si>
-    <t>G, H</t>
+    <t>7, 8</t>
   </si>
 </sst>
 </file>
@@ -494,7 +470,7 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L1" s="1"/>
       <c r="M1" s="2"/>
@@ -508,7 +484,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -523,11 +499,11 @@
       <c r="U2" s="3"/>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>3</v>
+      <c r="A3">
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -542,11 +518,11 @@
       <c r="U3" s="3"/>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
       </c>
       <c r="C4">
         <v>6</v>
@@ -561,11 +537,11 @@
       <c r="U4" s="3"/>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="A5">
         <v>3</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
       </c>
       <c r="C5">
         <v>4</v>
@@ -580,11 +556,11 @@
       <c r="U5" s="3"/>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="A6">
         <v>4</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
       </c>
       <c r="C6">
         <v>5</v>
@@ -599,11 +575,11 @@
       <c r="U6" s="3"/>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
-        <v>4</v>
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
       </c>
       <c r="C7">
         <v>10</v>
@@ -618,11 +594,11 @@
       <c r="U7" s="3"/>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="A8">
         <v>6</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
       </c>
       <c r="C8">
         <v>9</v>
@@ -637,11 +613,11 @@
       <c r="U8" s="3"/>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>11</v>
+      <c r="A9">
+        <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C9">
         <v>8</v>
@@ -656,11 +632,11 @@
       <c r="U9" s="3"/>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" t="s">
-        <v>9</v>
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>6</v>
       </c>
       <c r="C10">
         <v>3</v>
@@ -679,7 +655,7 @@
         <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C11">
         <v>0</v>

</xml_diff>